<commit_message>
Updated DEU model - 2025-09-07 02:26
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73C92B4B-2037-44B7-A541-59D30E3BB2E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FA510EB-8813-4E97-B341-700E6B724BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6866,7 +6866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A395AC52-6F77-410E-B691-62E42D941722}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E73A424-89F8-4FD5-B2FE-7E7D623DF9BF}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6948,7 +6948,7 @@
         <v>2.9460000000000002</v>
       </c>
       <c r="M11">
-        <v>0.16629043199999999</v>
+        <v>0.1662904323543602</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -6986,7 +6986,7 @@
         <v>0.3765</v>
       </c>
       <c r="M12">
-        <v>0.16605894099999999</v>
+        <v>0.1660589409575936</v>
       </c>
       <c r="N12">
         <v>4</v>
@@ -7024,7 +7024,7 @@
         <v>0.86850000000000005</v>
       </c>
       <c r="M13">
-        <v>0.166036871</v>
+        <v>0.16603687133815981</v>
       </c>
       <c r="N13">
         <v>2</v>
@@ -7062,7 +7062,7 @@
         <v>2.3174999999999999</v>
       </c>
       <c r="M14">
-        <v>0.166009988</v>
+        <v>0.16600998761152111</v>
       </c>
       <c r="N14">
         <v>3</v>
@@ -7100,7 +7100,7 @@
         <v>3.2130000000000001</v>
       </c>
       <c r="M15">
-        <v>0.15791618144117647</v>
+        <v>0.15791618136540428</v>
       </c>
       <c r="N15">
         <v>4</v>
@@ -7138,7 +7138,7 @@
         <v>15.913500000000001</v>
       </c>
       <c r="M16">
-        <v>0.15780781694895843</v>
+        <v>0.1578078168797811</v>
       </c>
       <c r="N16">
         <v>2</v>
@@ -7176,7 +7176,7 @@
         <v>0.30449999999999999</v>
       </c>
       <c r="M17">
-        <v>0.1576304955862069</v>
+        <v>0.15763049594795012</v>
       </c>
       <c r="N17">
         <v>5</v>
@@ -7214,7 +7214,7 @@
         <v>19.1175</v>
       </c>
       <c r="M18">
-        <v>0.15708286501294624</v>
+        <v>0.15708286511247102</v>
       </c>
       <c r="N18">
         <v>1</v>
@@ -7252,7 +7252,7 @@
         <v>17.7135</v>
       </c>
       <c r="M19">
-        <v>0.15591190081776607</v>
+        <v>0.1559119009051162</v>
       </c>
       <c r="N19">
         <v>3</v>
@@ -7290,7 +7290,7 @@
         <v>55.235250000000001</v>
       </c>
       <c r="M20">
-        <v>0.15242640939611934</v>
+        <v>0.15242640936734639</v>
       </c>
       <c r="N20">
         <v>1</v>
@@ -7328,7 +7328,7 @@
         <v>35.448749999999997</v>
       </c>
       <c r="M21">
-        <v>0.1492292388035967</v>
+        <v>0.14922923885275707</v>
       </c>
       <c r="N21">
         <v>4</v>
@@ -7366,7 +7366,7 @@
         <v>48.84675</v>
       </c>
       <c r="M22">
-        <v>0.14900018618331312</v>
+        <v>0.14900018618577154</v>
       </c>
       <c r="N22">
         <v>2</v>
@@ -7404,7 +7404,7 @@
         <v>37.276499999999999</v>
       </c>
       <c r="M23">
-        <v>0.14696908609122369</v>
+        <v>0.14696908603529971</v>
       </c>
       <c r="N23">
         <v>3</v>
@@ -7442,7 +7442,7 @@
         <v>30.28725</v>
       </c>
       <c r="M24">
-        <v>0.1464046198908204</v>
+        <v>0.14640461999321244</v>
       </c>
       <c r="N24">
         <v>5</v>
@@ -7480,7 +7480,7 @@
         <v>101.51625</v>
       </c>
       <c r="M25">
-        <v>0.14266988444631526</v>
+        <v>0.14266988441536055</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -7518,7 +7518,7 @@
         <v>103.524</v>
       </c>
       <c r="M26">
-        <v>0.13860597241461403</v>
+        <v>0.13860597249684553</v>
       </c>
       <c r="N26">
         <v>5</v>
@@ -7556,7 +7556,7 @@
         <v>97.376999999999995</v>
       </c>
       <c r="M27">
-        <v>0.13792351711269604</v>
+        <v>0.1379235172174148</v>
       </c>
       <c r="N27">
         <v>2</v>
@@ -7594,7 +7594,7 @@
         <v>103.755</v>
       </c>
       <c r="M28">
-        <v>0.13713528867831432</v>
+        <v>0.13713528865346272</v>
       </c>
       <c r="N28">
         <v>4</v>
@@ -7632,7 +7632,7 @@
         <v>88.663499999999999</v>
       </c>
       <c r="M29">
-        <v>0.13654150962306927</v>
+        <v>0.13654150960518857</v>
       </c>
       <c r="N29">
         <v>3</v>
@@ -7670,7 +7670,7 @@
         <v>83.819249999999997</v>
       </c>
       <c r="M30">
-        <v>0.13376983621610786</v>
+        <v>0.13376983623565916</v>
       </c>
       <c r="N30">
         <v>1</v>
@@ -7708,7 +7708,7 @@
         <v>63.249749999999999</v>
       </c>
       <c r="M31">
-        <v>0.13372190909688969</v>
+        <v>0.13372190917245153</v>
       </c>
       <c r="N31">
         <v>2</v>
@@ -7746,7 +7746,7 @@
         <v>65.268749999999997</v>
       </c>
       <c r="M32">
-        <v>0.13341965170718761</v>
+        <v>0.13341965150528012</v>
       </c>
       <c r="N32">
         <v>3</v>
@@ -7784,7 +7784,7 @@
         <v>72.006</v>
       </c>
       <c r="M33">
-        <v>0.13329939427113366</v>
+        <v>0.13329939427311402</v>
       </c>
       <c r="N33">
         <v>5</v>
@@ -7822,7 +7822,7 @@
         <v>71.385750000000002</v>
       </c>
       <c r="M34">
-        <v>0.13204864563094526</v>
+        <v>0.1320486454572623</v>
       </c>
       <c r="N34">
         <v>4</v>
@@ -7834,7 +7834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF049B48-9CC0-4CFE-ACF4-F9B56B3B83FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4A1F8B1-67F0-41A0-8C6F-CA296B34EB0B}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14736,7 +14736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01BBBAD1-33A4-4F25-940E-E70C475CA750}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B572E010-8CB7-41C2-A01D-25F1B3C3D8C0}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-07 18:57
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52486C56-C2AD-48C8-BC68-06B5C5DFFE5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2834FF70-F0A9-4433-B508-ED8293A4509C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6866,7 +6866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7314F02B-E03D-4979-8E2B-EE9344C32764}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C87FCBB-0CDA-4F98-8A31-58215B1DA76F}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7834,7 +7834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8E74485-4207-4546-BC54-D0DEAA9D4472}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C055281-58B2-46AB-97F2-C6B64ABC1F41}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14736,7 +14736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F1FE5DE-32CB-42D7-A81E-5353E2A0627D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4F9C7C-6206-42F3-A678-5C13ABF0B085}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-07 19:18
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2834FF70-F0A9-4433-B508-ED8293A4509C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B7DABF7-B4FF-413C-A7FF-709160ECDB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6866,7 +6866,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C87FCBB-0CDA-4F98-8A31-58215B1DA76F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17EB2D6B-0ABD-4C3A-AD10-739512ADB08E}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7834,7 +7834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C055281-58B2-46AB-97F2-C6B64ABC1F41}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4865EA13-E4D3-4648-95F1-BD77EF6AD29E}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14736,7 +14736,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4F9C7C-6206-42F3-A678-5C13ABF0B085}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38C3FCE1-F906-4899-8B4F-F7BB31F020E3}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-13 01:59
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9A852FD-C322-497A-975B-83EC6D939064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB9CE892-D6CB-45D5-B4C3-F794E4783D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DB8BC63-2AF8-49CD-8497-3720EC1DC224}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0BCDA2C-378A-497F-8655-1D6780CFEC81}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F873EBB2-581A-4E7A-ADD2-0E2E9693D571}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA2FCBD-F06F-4F04-A280-D369F617192A}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93D18FE2-B9FA-4B08-82A0-BB839B987C5D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{407D55C7-B3C4-4B35-8446-9C46A3D6AAB9}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-13 09:22
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB9CE892-D6CB-45D5-B4C3-F794E4783D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{16CE2550-A8D8-4C0C-A780-81C081B7B31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0BCDA2C-378A-497F-8655-1D6780CFEC81}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F601B599-0212-43B5-9463-6CB7FCC927A3}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA2FCBD-F06F-4F04-A280-D369F617192A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CFCEF70-2C7A-4BCF-A551-EAE833894953}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{407D55C7-B3C4-4B35-8446-9C46A3D6AAB9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C2FE76-4228-43BC-B24E-449586C0E33E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-13 10:03
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16CE2550-A8D8-4C0C-A780-81C081B7B31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{995A8853-7C57-45D4-95FB-B64DB31A34A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F601B599-0212-43B5-9463-6CB7FCC927A3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ABA850B-2276-49A3-99C2-C36210D13E31}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CFCEF70-2C7A-4BCF-A551-EAE833894953}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D67B224F-19F9-4706-91FB-3E51117914DA}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C2FE76-4228-43BC-B24E-449586C0E33E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073D65B1-BBDD-455E-8C64-6070E3D8E00E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-14 18:16
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{995A8853-7C57-45D4-95FB-B64DB31A34A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C10F4E5-FF03-4D81-A118-0248B478FA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ABA850B-2276-49A3-99C2-C36210D13E31}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A30E62-FFC4-488D-A311-12D5AB0AC9D3}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D67B224F-19F9-4706-91FB-3E51117914DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2C81906-CB01-4C85-B6EE-263BBC4A3D38}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073D65B1-BBDD-455E-8C64-6070E3D8E00E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03772941-7DA5-47C5-B97F-8179BF68A682}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-14 18:45
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C10F4E5-FF03-4D81-A118-0248B478FA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD3904CD-D950-4894-9E3B-335DC105E0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A30E62-FFC4-488D-A311-12D5AB0AC9D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809C680D-4511-49FB-B80C-6ADB2FD0EEF6}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2C81906-CB01-4C85-B6EE-263BBC4A3D38}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F51E90F-FB2E-495E-A3BA-539416544EBB}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03772941-7DA5-47C5-B97F-8179BF68A682}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A435E7-6347-4C93-9199-4E6E00D412CB}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-14 19:06
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD3904CD-D950-4894-9E3B-335DC105E0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FBC971A-D795-4D94-ACC6-AA55A4DCF589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6870,7 +6870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809C680D-4511-49FB-B80C-6ADB2FD0EEF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E929A3-A83E-4753-8254-B5CFA66A6C41}">
   <dimension ref="B9:N34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7838,7 +7838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F51E90F-FB2E-495E-A3BA-539416544EBB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BBCA2A3-316F-4A43-ACEF-60E25E43FE9D}">
   <dimension ref="B9:AB154"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14740,7 +14740,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A435E7-6347-4C93-9199-4E6E00D412CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C288B21D-C07A-4141-BCFE-FD737B71EE8E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-12-10 20:03
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF96098A-BAFC-4F66-A277-F4AA60A4B8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{78B8234A-0D4B-4F4A-9D54-939A35AF21C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="370">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -618,6 +618,9 @@
     <t>wnid offshore potential</t>
   </si>
   <si>
+    <t>ELC_BatIn</t>
+  </si>
+  <si>
     <t>~fi_process</t>
   </si>
   <si>
@@ -1231,6 +1234,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>e_DE62-380,e_w170123812-400,e_w59026005-380,e_w952346322-380</t>
   </si>
 </sst>
 </file>
@@ -3124,7 +3130,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_DE62-380,e_w170123812-400,e_w59026005-380,e_w952346322-380</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3146,7 +3152,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_DE62-380,e_w170123812-400,e_w59026005-380,e_w952346322-380</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3161,7 +3167,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>19</v>
+        <v>369</v>
       </c>
     </row>
   </sheetData>
@@ -4638,9 +4644,8 @@
     <row r="8" spans="2:25" ht="17.649999999999999">
       <c r="B8" s="20"/>
       <c r="E8" s="26"/>
-      <c r="F8" t="str">
-        <f>C5</f>
-        <v>ELC</v>
+      <c r="F8" t="s">
+        <v>163</v>
       </c>
       <c r="G8" t="str">
         <f>E7</f>
@@ -5963,62 +5968,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AFE63CA-8333-4676-B1D1-2E22E36AA8F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{649865C8-F8BF-49DB-831B-5C407E3D9476}">
   <dimension ref="B9:M33"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:13">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
-        <v>167</v>
-      </c>
-      <c r="F10" t="s">
-        <v>168</v>
-      </c>
-      <c r="G10" t="s">
-        <v>169</v>
-      </c>
-      <c r="H10" t="s">
-        <v>170</v>
-      </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
       <c r="K10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="L10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6027,16 +6032,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L11">
         <v>13.938003670888978</v>
@@ -6047,13 +6052,13 @@
     </row>
     <row r="12" spans="2:13">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -6062,16 +6067,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L12">
         <v>18.31863654586293</v>
@@ -6082,13 +6087,13 @@
     </row>
     <row r="13" spans="2:13">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -6097,16 +6102,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L13">
         <v>30.238043484360141</v>
@@ -6117,13 +6122,13 @@
     </row>
     <row r="14" spans="2:13">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -6132,16 +6137,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L14">
         <v>45.351574205977535</v>
@@ -6152,13 +6157,13 @@
     </row>
     <row r="15" spans="2:13">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -6167,16 +6172,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L15">
         <v>34.531914591504368</v>
@@ -6187,13 +6192,13 @@
     </row>
     <row r="16" spans="2:13">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -6202,16 +6207,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="L16">
         <v>38.190379780391297</v>
@@ -6222,13 +6227,13 @@
     </row>
     <row r="17" spans="2:13">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -6237,16 +6242,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K17" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L17">
         <v>13.44361680351453</v>
@@ -6257,13 +6262,13 @@
     </row>
     <row r="18" spans="2:13">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -6272,16 +6277,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="L18">
         <v>15.833691242733796</v>
@@ -6292,13 +6297,13 @@
     </row>
     <row r="19" spans="2:13">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -6307,16 +6312,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L19">
         <v>11.346394535605524</v>
@@ -6327,13 +6332,13 @@
     </row>
     <row r="20" spans="2:13">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -6342,16 +6347,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L20">
         <v>32.21637396151899</v>
@@ -6362,13 +6367,13 @@
     </row>
     <row r="21" spans="2:13">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -6377,16 +6382,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K21" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L21">
         <v>30.007867954603132</v>
@@ -6397,13 +6402,13 @@
     </row>
     <row r="22" spans="2:13">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -6412,16 +6417,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L22">
         <v>38.24309918267349</v>
@@ -6432,13 +6437,13 @@
     </row>
     <row r="23" spans="2:13">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -6447,16 +6452,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L23">
         <v>0.95743993217852441</v>
@@ -6467,13 +6472,13 @@
     </row>
     <row r="24" spans="2:13">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -6482,16 +6487,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L24">
         <v>15.746380528104394</v>
@@ -6502,13 +6507,13 @@
     </row>
     <row r="25" spans="2:13">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -6517,16 +6522,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L25">
         <v>32.685256480874017</v>
@@ -6537,13 +6542,13 @@
     </row>
     <row r="26" spans="2:13">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -6552,16 +6557,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K26" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L26">
         <v>13.348518217290337</v>
@@ -6572,13 +6577,13 @@
     </row>
     <row r="27" spans="2:13">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -6587,16 +6592,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K27" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L27">
         <v>19.75277137741244</v>
@@ -6607,13 +6612,13 @@
     </row>
     <row r="28" spans="2:13">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D28" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -6622,16 +6627,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L28">
         <v>23.3954191787236</v>
@@ -6642,13 +6647,13 @@
     </row>
     <row r="29" spans="2:13">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D29" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -6657,16 +6662,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K29" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="L29">
         <v>20.01197763203729</v>
@@ -6677,13 +6682,13 @@
     </row>
     <row r="30" spans="2:13">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -6692,16 +6697,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K30" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L30">
         <v>23.591873553963495</v>
@@ -6712,13 +6717,13 @@
     </row>
     <row r="31" spans="2:13">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D31" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -6727,16 +6732,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K31" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L31">
         <v>21.653826323424543</v>
@@ -6747,13 +6752,13 @@
     </row>
     <row r="32" spans="2:13">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -6762,16 +6767,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L32">
         <v>12.637613221312568</v>
@@ -6782,13 +6787,13 @@
     </row>
     <row r="33" spans="2:13">
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -6797,16 +6802,16 @@
         <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L33">
         <v>23.28078369016097</v>
@@ -6821,101 +6826,101 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF16C26-3322-4C07-9407-08FCC9B13B83}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367102E2-9D51-4C63-98B2-4FFE82EE758D}">
   <dimension ref="B9:Z32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:26">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="W9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="2:26">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
+        <v>166</v>
+      </c>
+      <c r="K10" t="s">
+        <v>222</v>
+      </c>
+      <c r="L10" t="s">
+        <v>223</v>
+      </c>
+      <c r="M10" t="s">
+        <v>224</v>
+      </c>
+      <c r="O10" t="s">
         <v>165</v>
       </c>
-      <c r="D10" t="s">
+      <c r="P10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
+      <c r="Q10" t="s">
         <v>167</v>
       </c>
-      <c r="F10" t="s">
+      <c r="R10" t="s">
         <v>168</v>
       </c>
-      <c r="G10" t="s">
+      <c r="S10" t="s">
         <v>169</v>
       </c>
-      <c r="H10" t="s">
+      <c r="T10" t="s">
         <v>170</v>
       </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
-      <c r="K10" t="s">
-        <v>221</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="U10" t="s">
+        <v>171</v>
+      </c>
+      <c r="W10" t="s">
+        <v>166</v>
+      </c>
+      <c r="X10" t="s">
         <v>222</v>
       </c>
-      <c r="M10" t="s">
+      <c r="Y10" t="s">
         <v>223</v>
       </c>
-      <c r="O10" t="s">
-        <v>164</v>
-      </c>
-      <c r="P10" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>166</v>
-      </c>
-      <c r="R10" t="s">
-        <v>167</v>
-      </c>
-      <c r="S10" t="s">
-        <v>168</v>
-      </c>
-      <c r="T10" t="s">
-        <v>169</v>
-      </c>
-      <c r="U10" t="s">
-        <v>170</v>
-      </c>
-      <c r="W10" t="s">
-        <v>165</v>
-      </c>
-      <c r="X10" t="s">
-        <v>221</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>222</v>
-      </c>
       <c r="Z10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="2:26">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6924,16 +6929,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L11">
         <v>79.362778177778793</v>
@@ -6942,13 +6947,13 @@
         <v>0.32113557799809911</v>
       </c>
       <c r="O11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="Q11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="R11" t="s">
         <v>10</v>
@@ -6957,16 +6962,16 @@
         <v>21</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="X11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Y11">
         <v>108.8275</v>
@@ -6977,13 +6982,13 @@
     </row>
     <row r="12" spans="2:26">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D12" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -6992,16 +6997,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K12" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L12">
         <v>50.354564381123943</v>
@@ -7010,13 +7015,13 @@
         <v>0.26229547814325971</v>
       </c>
       <c r="O12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Q12" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="R12" t="s">
         <v>10</v>
@@ -7025,16 +7030,16 @@
         <v>21</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="X12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="Y12">
         <v>54.292499999999997</v>
@@ -7045,13 +7050,13 @@
     </row>
     <row r="13" spans="2:26">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -7060,16 +7065,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L13">
         <v>57.005439523831519</v>
@@ -7078,13 +7083,13 @@
         <v>0.27008680004560909</v>
       </c>
       <c r="O13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Q13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="R13" t="s">
         <v>10</v>
@@ -7093,16 +7098,16 @@
         <v>21</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="X13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Y13">
         <v>50.356250000000003</v>
@@ -7113,13 +7118,13 @@
     </row>
     <row r="14" spans="2:26">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -7128,16 +7133,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L14">
         <v>19.895723562817633</v>
@@ -7146,13 +7151,13 @@
         <v>0.41998320074620132</v>
       </c>
       <c r="O14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R14" t="s">
         <v>10</v>
@@ -7161,16 +7166,16 @@
         <v>21</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="X14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="Y14">
         <v>9.5987500000000008</v>
@@ -7181,13 +7186,13 @@
     </row>
     <row r="15" spans="2:26">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -7196,16 +7201,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L15">
         <v>9.5699994650614961</v>
@@ -7214,13 +7219,13 @@
         <v>0.44653362265814228</v>
       </c>
       <c r="O15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q15" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="R15" t="s">
         <v>10</v>
@@ -7229,16 +7234,16 @@
         <v>21</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="X15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="Y15">
         <v>50.66</v>
@@ -7249,13 +7254,13 @@
     </row>
     <row r="16" spans="2:26">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D16" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -7264,16 +7269,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K16" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L16">
         <v>44.760252416795389</v>
@@ -7282,13 +7287,13 @@
         <v>0.42821243398456738</v>
       </c>
       <c r="O16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P16" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="Q16" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="R16" t="s">
         <v>10</v>
@@ -7297,16 +7302,16 @@
         <v>21</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W16" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="X16" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="Y16">
         <v>5.0000000000000001E-3</v>
@@ -7317,13 +7322,13 @@
     </row>
     <row r="17" spans="2:26">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -7332,16 +7337,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="K17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L17">
         <v>40.59880776523103</v>
@@ -7350,13 +7355,13 @@
         <v>0.34199104865897728</v>
       </c>
       <c r="O17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="Q17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="R17" t="s">
         <v>10</v>
@@ -7365,16 +7370,16 @@
         <v>21</v>
       </c>
       <c r="T17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="X17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="Y17">
         <v>0.92625000000000002</v>
@@ -7385,13 +7390,13 @@
     </row>
     <row r="18" spans="2:26">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D18" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -7400,16 +7405,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L18">
         <v>71.045385513132985</v>
@@ -7418,13 +7423,13 @@
         <v>0.30696999602332747</v>
       </c>
       <c r="O18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="R18" t="s">
         <v>10</v>
@@ -7433,16 +7438,16 @@
         <v>21</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="X18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Y18">
         <v>7.5287499999999996</v>
@@ -7453,13 +7458,13 @@
     </row>
     <row r="19" spans="2:26">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -7468,16 +7473,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K19" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L19">
         <v>63.055598832310729</v>
@@ -7486,13 +7491,13 @@
         <v>0.3285833519844587</v>
       </c>
       <c r="O19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P19" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q19" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="R19" t="s">
         <v>10</v>
@@ -7501,16 +7506,16 @@
         <v>21</v>
       </c>
       <c r="T19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W19" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="X19" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Y19">
         <v>14.6</v>
@@ -7521,13 +7526,13 @@
     </row>
     <row r="20" spans="2:26">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D20" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -7536,16 +7541,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K20" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L20">
         <v>43.89469200396065</v>
@@ -7554,13 +7559,13 @@
         <v>0.2838221752225063</v>
       </c>
       <c r="O20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P20" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q20" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="R20" t="s">
         <v>10</v>
@@ -7569,16 +7574,16 @@
         <v>21</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W20" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X20" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="Y20">
         <v>0.24374999999999999</v>
@@ -7589,13 +7594,13 @@
     </row>
     <row r="21" spans="2:26">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -7604,16 +7609,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K21" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L21">
         <v>11.547936358898198</v>
@@ -7624,13 +7629,13 @@
     </row>
     <row r="22" spans="2:26">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -7639,16 +7644,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K22" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L22">
         <v>31.481356456094364</v>
@@ -7659,13 +7664,13 @@
     </row>
     <row r="23" spans="2:26">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D23" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -7674,16 +7679,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="K23" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L23">
         <v>15.708789779919334</v>
@@ -7694,13 +7699,13 @@
     </row>
     <row r="24" spans="2:26">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -7709,16 +7714,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K24" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L24">
         <v>20.814752751471318</v>
@@ -7729,13 +7734,13 @@
     </row>
     <row r="25" spans="2:26">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D25" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -7744,16 +7749,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K25" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L25">
         <v>50.266717026070005</v>
@@ -7764,13 +7769,13 @@
     </row>
     <row r="26" spans="2:26">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D26" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -7779,16 +7784,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K26" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L26">
         <v>56.728889145623882</v>
@@ -7799,13 +7804,13 @@
     </row>
     <row r="27" spans="2:26">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -7814,16 +7819,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="K27" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L27">
         <v>70.602917671125681</v>
@@ -7834,13 +7839,13 @@
     </row>
     <row r="28" spans="2:26">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D28" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -7849,16 +7854,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K28" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L28">
         <v>7.8153674765988201</v>
@@ -7869,13 +7874,13 @@
     </row>
     <row r="29" spans="2:26">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D29" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -7884,16 +7889,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K29" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L29">
         <v>26.861604762024118</v>
@@ -7904,13 +7909,13 @@
     </row>
     <row r="30" spans="2:26">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D30" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -7919,16 +7924,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="K30" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L30">
         <v>10.889866530825216</v>
@@ -7939,13 +7944,13 @@
     </row>
     <row r="31" spans="2:26">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D31" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -7954,16 +7959,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L31">
         <v>9.0084683548455349</v>
@@ -7974,13 +7979,13 @@
     </row>
     <row r="32" spans="2:26">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -7989,16 +7994,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K32" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L32">
         <v>35.009005865752776</v>
@@ -8013,27 +8018,27 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA7EECA8-DDEF-461B-BE98-FA221DB124DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72517389-39D8-45BF-BB64-2955DEEA03F5}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:16">
       <c r="B9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:16">
       <c r="B10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E10">
         <v>2023</v>
@@ -8048,30 +8053,30 @@
         <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="2:16">
       <c r="B11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -8092,10 +8097,10 @@
         <v>146</v>
       </c>
       <c r="J11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
@@ -8104,15 +8109,15 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="12" spans="2:16">
       <c r="B12" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -8130,13 +8135,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H12" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K12" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
@@ -8145,15 +8150,15 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P12" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="13" spans="2:16">
       <c r="B13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
@@ -8171,13 +8176,13 @@
         <v>5100</v>
       </c>
       <c r="H13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K13" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M13" t="s">
         <v>10</v>
@@ -8186,15 +8191,15 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P13" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="B14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -8212,13 +8217,13 @@
         <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="M14" t="s">
         <v>10</v>
@@ -8227,15 +8232,15 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P14" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -8253,13 +8258,13 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K15" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="M15" t="s">
         <v>10</v>
@@ -8268,15 +8273,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P15" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="16" spans="2:16">
       <c r="B16" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -8297,10 +8302,10 @@
         <v>146</v>
       </c>
       <c r="J16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K16" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="M16" t="s">
         <v>10</v>
@@ -8309,15 +8314,15 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P16" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -8335,13 +8340,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K17" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="M17" t="s">
         <v>10</v>
@@ -8350,15 +8355,15 @@
         <v>21</v>
       </c>
       <c r="O17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -8376,13 +8381,13 @@
         <v>2300</v>
       </c>
       <c r="H18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="M18" t="s">
         <v>10</v>
@@ -8391,15 +8396,15 @@
         <v>21</v>
       </c>
       <c r="O18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="B19" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -8417,13 +8422,13 @@
         <v>80</v>
       </c>
       <c r="H19" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K19" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M19" t="s">
         <v>10</v>
@@ -8432,15 +8437,15 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P19" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="B20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
@@ -8458,13 +8463,13 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K20" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="M20" t="s">
         <v>10</v>
@@ -8473,15 +8478,15 @@
         <v>21</v>
       </c>
       <c r="O20" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P20" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -8502,10 +8507,10 @@
         <v>146</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K21" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="M21" t="s">
         <v>10</v>
@@ -8514,15 +8519,15 @@
         <v>21</v>
       </c>
       <c r="O21" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P21" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C22" t="s">
         <v>33</v>
@@ -8540,13 +8545,13 @@
         <v>1000</v>
       </c>
       <c r="H22" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="M22" t="s">
         <v>10</v>
@@ -8555,15 +8560,15 @@
         <v>21</v>
       </c>
       <c r="O22" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P22" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -8581,13 +8586,13 @@
         <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K23" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="M23" t="s">
         <v>10</v>
@@ -8596,15 +8601,15 @@
         <v>21</v>
       </c>
       <c r="O23" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P23" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="24" spans="2:16">
       <c r="B24" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C24" t="s">
         <v>33</v>
@@ -8625,10 +8630,10 @@
         <v>146</v>
       </c>
       <c r="J24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K24" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M24" t="s">
         <v>10</v>
@@ -8637,15 +8642,15 @@
         <v>21</v>
       </c>
       <c r="O24" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P24" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="25" spans="2:16">
       <c r="B25" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -8663,13 +8668,13 @@
         <v>2400</v>
       </c>
       <c r="H25" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="J25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K25" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M25" t="s">
         <v>10</v>
@@ -8678,15 +8683,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="26" spans="2:16">
       <c r="B26" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C26" t="s">
         <v>33</v>
@@ -8704,13 +8709,13 @@
         <v>60</v>
       </c>
       <c r="H26" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K26" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="M26" t="s">
         <v>10</v>
@@ -8719,15 +8724,15 @@
         <v>21</v>
       </c>
       <c r="O26" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P26" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" spans="2:16">
       <c r="B27" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -8748,10 +8753,10 @@
         <v>146</v>
       </c>
       <c r="J27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="M27" t="s">
         <v>10</v>
@@ -8760,15 +8765,15 @@
         <v>21</v>
       </c>
       <c r="O27" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P27" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="28" spans="2:16">
       <c r="B28" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -8786,12 +8791,12 @@
         <v>4350</v>
       </c>
       <c r="H28" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -8809,12 +8814,12 @@
         <v>130</v>
       </c>
       <c r="H29" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="B30" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
@@ -8837,7 +8842,7 @@
     </row>
     <row r="31" spans="2:16">
       <c r="B31" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C31" t="s">
         <v>33</v>
@@ -8855,12 +8860,12 @@
         <v>500</v>
       </c>
       <c r="H31" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="B32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C32" t="s">
         <v>33</v>
@@ -8878,12 +8883,12 @@
         <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
@@ -8906,7 +8911,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
@@ -8924,12 +8929,12 @@
         <v>0.35000000000000003</v>
       </c>
       <c r="H34" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -8947,12 +8952,12 @@
         <v>2650</v>
       </c>
       <c r="H35" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -8970,12 +8975,12 @@
         <v>65</v>
       </c>
       <c r="H36" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -8993,12 +8998,12 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -9021,7 +9026,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -9039,12 +9044,12 @@
         <v>2300</v>
       </c>
       <c r="H39" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -9062,12 +9067,12 @@
         <v>80</v>
       </c>
       <c r="H40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -9090,7 +9095,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C42" t="s">
         <v>32</v>
@@ -9108,12 +9113,12 @@
         <v>5100</v>
       </c>
       <c r="H42" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -9131,12 +9136,12 @@
         <v>180</v>
       </c>
       <c r="H43" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C44" t="s">
         <v>36</v>
@@ -9159,7 +9164,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C45" t="s">
         <v>36</v>
@@ -9177,12 +9182,12 @@
         <v>4500</v>
       </c>
       <c r="H45" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C46" t="s">
         <v>36</v>
@@ -9200,12 +9205,12 @@
         <v>160</v>
       </c>
       <c r="H46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
@@ -9228,7 +9233,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
@@ -9246,12 +9251,12 @@
         <v>5100</v>
       </c>
       <c r="H48" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C49" t="s">
         <v>32</v>
@@ -9269,12 +9274,12 @@
         <v>155</v>
       </c>
       <c r="H49" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -9297,7 +9302,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -9315,12 +9320,12 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H51" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
@@ -9338,12 +9343,12 @@
         <v>340</v>
       </c>
       <c r="H52" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C53" t="s">
         <v>27</v>
@@ -9361,12 +9366,12 @@
         <v>10</v>
       </c>
       <c r="H53" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="B54" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C54" t="s">
         <v>27</v>
@@ -9384,12 +9389,12 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="B55" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C55" t="s">
         <v>32</v>
@@ -9412,7 +9417,7 @@
     </row>
     <row r="56" spans="2:8">
       <c r="B56" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
@@ -9430,12 +9435,12 @@
         <v>1700</v>
       </c>
       <c r="H56" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="B57" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C57" t="s">
         <v>32</v>
@@ -9453,12 +9458,12 @@
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="B58" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C58" t="s">
         <v>32</v>
@@ -9481,7 +9486,7 @@
     </row>
     <row r="59" spans="2:8">
       <c r="B59" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
@@ -9499,12 +9504,12 @@
         <v>2000</v>
       </c>
       <c r="H59" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="B60" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -9522,12 +9527,12 @@
         <v>60</v>
       </c>
       <c r="H60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="B61" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C61" t="s">
         <v>32</v>
@@ -9550,7 +9555,7 @@
     </row>
     <row r="62" spans="2:8">
       <c r="B62" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C62" t="s">
         <v>32</v>
@@ -9568,12 +9573,12 @@
         <v>2200</v>
       </c>
       <c r="H62" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="B63" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -9591,15 +9596,15 @@
         <v>65</v>
       </c>
       <c r="H63" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="64" spans="2:8">
       <c r="B64" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C64" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D64" t="s">
         <v>19</v>
@@ -9619,10 +9624,10 @@
     </row>
     <row r="65" spans="2:8">
       <c r="B65" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C65" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D65" t="s">
         <v>19</v>
@@ -9637,15 +9642,15 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H65" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="66" spans="2:8">
       <c r="B66" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C66" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D66" t="s">
         <v>19</v>
@@ -9660,15 +9665,15 @@
         <v>1660</v>
       </c>
       <c r="H66" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C67" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D67" t="s">
         <v>19</v>
@@ -9683,15 +9688,15 @@
         <v>40</v>
       </c>
       <c r="H67" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C68" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -9706,15 +9711,15 @@
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" t="s">
+        <v>366</v>
+      </c>
+      <c r="C69" t="s">
         <v>365</v>
-      </c>
-      <c r="C69" t="s">
-        <v>364</v>
       </c>
       <c r="D69" t="s">
         <v>19</v>
@@ -9734,10 +9739,10 @@
     </row>
     <row r="70" spans="2:8">
       <c r="B70" t="s">
+        <v>366</v>
+      </c>
+      <c r="C70" t="s">
         <v>365</v>
-      </c>
-      <c r="C70" t="s">
-        <v>364</v>
       </c>
       <c r="D70" t="s">
         <v>19</v>
@@ -9752,15 +9757,15 @@
         <v>0.3</v>
       </c>
       <c r="H70" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="B71" t="s">
+        <v>366</v>
+      </c>
+      <c r="C71" t="s">
         <v>365</v>
-      </c>
-      <c r="C71" t="s">
-        <v>364</v>
       </c>
       <c r="D71" t="s">
         <v>19</v>
@@ -9775,15 +9780,15 @@
         <v>1490</v>
       </c>
       <c r="H71" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="B72" t="s">
+        <v>366</v>
+      </c>
+      <c r="C72" t="s">
         <v>365</v>
-      </c>
-      <c r="C72" t="s">
-        <v>364</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
@@ -9798,15 +9803,15 @@
         <v>38</v>
       </c>
       <c r="H72" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="B73" t="s">
+        <v>366</v>
+      </c>
+      <c r="C73" t="s">
         <v>365</v>
-      </c>
-      <c r="C73" t="s">
-        <v>364</v>
       </c>
       <c r="D73" t="s">
         <v>19</v>
@@ -9821,7 +9826,7 @@
         <v>1.5</v>
       </c>
       <c r="H73" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated DEU model - 2025-12-11 09:36
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_DEU/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78B8234A-0D4B-4F4A-9D54-939A35AF21C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F04EAA67-405A-4CA3-A871-DBF9F31662A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5968,7 +5968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{649865C8-F8BF-49DB-831B-5C407E3D9476}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{446257EC-88C4-4692-B573-238A2AC055B1}">
   <dimension ref="B9:M33"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6826,7 +6826,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367102E2-9D51-4C63-98B2-4FFE82EE758D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E33203C-464F-4769-8E89-FC85B1B64F3F}">
   <dimension ref="B9:Z32"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8018,7 +8018,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72517389-39D8-45BF-BB64-2955DEEA03F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8335C02-94C5-4A09-AA03-D3E81F945F89}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>